<commit_message>
Reorganize: move 37 articles to blog/ subdirectory, add scraper pipeline
- Move all article HTML pages from root into blog/ for a clean root directory
- Switch vite.config.js base from './' to '/' (required for subdirectory pages)
- Update build-components.js to use absolute paths in nav/JS injection and scan blog/ dir
- Patch all article files: absolute CSS/JS paths, /blog.html back-links, blog/ canonical URLs
- Update blog.html cards, resources.html, case-studies.html, templates-tools.html links
- Update sync-blog.js, generate-sitemap.js, .pa11yci.json for blog/ paths
- Add all 30 new articles to sitemap and pa11yci (were missing)
- Fix: manifest.json moved to public/ (was missing from Vite build output)
- Fix: lighthouse-budget.json moved to tools/testing/ (was orphaned at root)
- Add blog content pipeline: scraper-admin.html, scraper-server.js, sync-blog.js, rss-feeds.json
- Update CLAUDE.md to reflect new structure

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Blog and Article Content/Articles.xlsx
+++ b/Blog and Article Content/Articles.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4BA0D45-8B80-401C-B880-6DF1AC35461A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Articles" state="visible" r:id="rId4"/>
+    <sheet name="Articles" sheetId="1" r:id="rId1"/>
+    <sheet name="Original" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="121">
   <si>
     <t>Source URL</t>
   </si>
@@ -229,7 +234,7 @@
     <t>Thu, 12 Feb 2026 17:56:11 +0000</t>
   </si>
   <si>
-    <t xml:space="preserve">Show your org some love: Strengthen your Salesforce security strategy.
+    <t>Show your org some love: Strengthen your Salesforce security strategy.
 The post 7 Reasons We Love Salesforce Security (And You Should Too!) appeared first on Cloud for Good.</t>
   </si>
   <si>
@@ -242,7 +247,7 @@
     <t>Tue, 10 Feb 2026 23:30:35 +0000</t>
   </si>
   <si>
-    <t xml:space="preserve">We are seeking a highly skilled and motivated AI Engineer to join our team in developing reusable AI-powered tools and components that drive automation, scalability, and efficiency across our
+    <t>We are seeking a highly skilled and motivated AI Engineer to join our team in developing reusable AI-powered tools and components that drive automation, scalability, and efficiency across our
 The post Senior AI Developer – Innovation Hub in India appeared first on Cloud for Good.</t>
   </si>
   <si>
@@ -258,7 +263,7 @@
     <t>Tue, 10 Feb 2026 23:26:20 +0000</t>
   </si>
   <si>
-    <t xml:space="preserve">The Senior Salesforce Developer will be a leading technical resource on the Salesforce implementation team. They will be responsible for evaluating, designing, and building key technical components
+    <t>The Senior Salesforce Developer will be a leading technical resource on the Salesforce implementation team. They will be responsible for evaluating, designing, and building key technical components
 The post Senior Salesforce Developer – Innovation Hub in India appeared first on Cloud for Good.</t>
   </si>
   <si>
@@ -274,7 +279,7 @@
     <t>Wed, 25 Mar 2026 01:02:30 +0000</t>
   </si>
   <si>
-    <t xml:space="preserve">As new work requirements for SNAP lurch into effect across the country, food banks and pantries are doing what they can to ease the blow. The timing of the new rules varies by state, but the upshot is that millions more Americans who previously qualified for SNAP will have to…
+    <t>As new work requirements for SNAP lurch into effect across the country, food banks and pantries are doing what they can to ease the blow. The timing of the new rules varies by state, but the upshot is that millions more Americans who previously qualified for SNAP will have to…
 The post SNAP Work Req</t>
   </si>
   <si>
@@ -305,7 +310,7 @@
     <t>Fri, 20 Mar 2026 14:24:10 +0000</t>
   </si>
   <si>
-    <t xml:space="preserve">After only one year of having a nutrition policy, Ferndale Food Bank of Washington state can’t imagine operating without one. Getting a nutrition policy in place went hand in hand with maturing from a very small operation into one that now serves nearly 300 people a week. As demand grew,…
+    <t>After only one year of having a nutrition policy, Ferndale Food Bank of Washington state can’t imagine operating without one. Getting a nutrition policy in place went hand in hand with maturing from a very small operation into one that now serves nearly 300 people a week. As demand grew,…
 The post P</t>
   </si>
   <si>
@@ -331,7 +336,7 @@
     <t>Tue, 10 Mar 2026 21:15:48 +0000</t>
   </si>
   <si>
-    <t xml:space="preserve">Food Bank of Eastern Oklahoma was known years ago for having the first production kitchen in the Feeding America network. “We had the first, but we were way behind in what we were doing with it,” noted Jeff Marlow, Chief Executive Officer.  That’s no longer the case, with a recent…
+    <t>Food Bank of Eastern Oklahoma was known years ago for having the first production kitchen in the Feeding America network. “We had the first, but we were way behind in what we were doing with it,” noted Jeff Marlow, Chief Executive Officer.  That’s no longer the case, with a recent…
 The post Food Ban</t>
   </si>
   <si>
@@ -356,7 +361,7 @@
     <t>Tue, 10 Mar 2026 01:34:30 +0000</t>
   </si>
   <si>
-    <t xml:space="preserve">Vinnie Oakes used to order produce by the case. Now he buys it by the truckload. That is just one of the differences Oakes encountered when he moved from a long career in restaurant and casino hospitality to Reno-based Food Bank of Northern Nevada, where he has served as Director…
+    <t>Vinnie Oakes used to order produce by the case. Now he buys it by the truckload. That is just one of the differences Oakes encountered when he moved from a long career in restaurant and casino hospitality to Reno-based Food Bank of Northern Nevada, where he has served as Director…
 The post From Casi</t>
   </si>
   <si>
@@ -369,7 +374,7 @@
     <t>Wed, 25 Feb 2026 14:52:22 +0000</t>
   </si>
   <si>
-    <t xml:space="preserve">Many people working in hunger relief lament the difficulty of eliminating hunger, a problem that seems like it should be easily resolved, given the world of plenty that we live in. But few respond to the issue by taking on a global research project involving travel to more than 90…
+    <t>Many people working in hunger relief lament the difficulty of eliminating hunger, a problem that seems like it should be easily resolved, given the world of plenty that we live in. But few respond to the issue by taking on a global research project involving travel to more than 90…
 The post Book Rev</t>
   </si>
   <si>
@@ -388,18 +393,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -429,15 +444,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -774,9 +793,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K24"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
@@ -789,7 +808,7 @@
     <col min="10" max="11" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -824,8 +843,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -860,7 +878,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -895,7 +913,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -930,7 +948,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
@@ -965,7 +983,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -1000,7 +1018,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>45</v>
       </c>
@@ -1035,7 +1053,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>51</v>
       </c>
@@ -1070,7 +1088,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>57</v>
       </c>
@@ -1105,7 +1123,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>61</v>
       </c>
@@ -1140,7 +1158,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>65</v>
       </c>
@@ -1175,7 +1193,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>69</v>
       </c>
@@ -1210,7 +1228,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>73</v>
       </c>
@@ -1245,7 +1263,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>78</v>
       </c>
@@ -1280,7 +1298,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>82</v>
       </c>
@@ -1315,7 +1333,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>88</v>
       </c>
@@ -1350,8 +1368,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
         <v>93</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -1385,8 +1403,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
         <v>97</v>
       </c>
       <c r="B19" t="s">
@@ -1420,7 +1438,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>101</v>
       </c>
@@ -1455,7 +1473,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>105</v>
       </c>
@@ -1490,7 +1508,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>109</v>
       </c>
@@ -1525,7 +1543,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>113</v>
       </c>
@@ -1560,7 +1578,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>117</v>
       </c>
@@ -1596,7 +1614,842 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A18" r:id="rId1" xr:uid="{166EDA43-6A69-41B3-B1A1-92E42F4C084B}"/>
+    <hyperlink ref="A19" r:id="rId2" xr:uid="{DEB7976F-DC21-4789-A5E0-2E7568AA06EE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67B11DAD-F541-46D1-8FB0-79FDB6722BD1}">
+  <dimension ref="A1:K24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="80" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="100" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="11" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" t="s">
+        <v>44</v>
+      </c>
+      <c r="I7" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9" t="s">
+        <v>56</v>
+      </c>
+      <c r="I9" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
+        <v>64</v>
+      </c>
+      <c r="H11" t="s">
+        <v>56</v>
+      </c>
+      <c r="I11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" t="s">
+        <v>30</v>
+      </c>
+      <c r="G13" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" t="s">
+        <v>56</v>
+      </c>
+      <c r="I13" t="s">
+        <v>19</v>
+      </c>
+      <c r="J13" t="s">
+        <v>20</v>
+      </c>
+      <c r="K13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" t="s">
+        <v>30</v>
+      </c>
+      <c r="G15" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" t="s">
+        <v>56</v>
+      </c>
+      <c r="I15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" t="s">
+        <v>91</v>
+      </c>
+      <c r="H17" t="s">
+        <v>92</v>
+      </c>
+      <c r="I17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" t="s">
+        <v>100</v>
+      </c>
+      <c r="H19" t="s">
+        <v>87</v>
+      </c>
+      <c r="I19" t="s">
+        <v>19</v>
+      </c>
+      <c r="J19" t="s">
+        <v>20</v>
+      </c>
+      <c r="K19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" t="s">
+        <v>106</v>
+      </c>
+      <c r="C21" t="s">
+        <v>84</v>
+      </c>
+      <c r="D21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" t="s">
+        <v>108</v>
+      </c>
+      <c r="H21" t="s">
+        <v>87</v>
+      </c>
+      <c r="I21" t="s">
+        <v>19</v>
+      </c>
+      <c r="J21" t="s">
+        <v>20</v>
+      </c>
+      <c r="K21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" t="s">
+        <v>84</v>
+      </c>
+      <c r="D23" t="s">
+        <v>115</v>
+      </c>
+      <c r="E23" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" t="s">
+        <v>116</v>
+      </c>
+      <c r="H23" t="s">
+        <v>92</v>
+      </c>
+      <c r="I23" t="s">
+        <v>19</v>
+      </c>
+      <c r="J23" t="s">
+        <v>20</v>
+      </c>
+      <c r="K23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A18" r:id="rId1" xr:uid="{F7384B20-C68C-4C74-A3B1-D49491D5F7B6}"/>
+    <hyperlink ref="A19" r:id="rId2" xr:uid="{979CF4F8-96F5-4302-9B67-0A1D9D7A46AA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>